<commit_message>
Atualiza eventos e dados das ligas
</commit_message>
<xml_diff>
--- a/2x2 online.xlsx
+++ b/2x2 online.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edd\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Edd\Desktop\Codes\Liga preconauta\preconauta-league\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D0E3281-0534-454A-982D-A174D661879D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E78BAB-C682-4E58-B304-E8684CCE7B4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4A5CD5E0-FAB5-4BBA-A2E8-DFE09CF06437}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="244">
   <si>
     <t>evento</t>
   </si>
@@ -675,6 +675,102 @@
   </si>
   <si>
     <t>Family Matters</t>
+  </si>
+  <si>
+    <t>Metusa &amp; Chueiry</t>
+  </si>
+  <si>
+    <t>Metusa</t>
+  </si>
+  <si>
+    <t>Massacre dos Maestros</t>
+  </si>
+  <si>
+    <t>Bell &amp; Greowtty</t>
+  </si>
+  <si>
+    <t>Bell</t>
+  </si>
+  <si>
+    <t>Greowtty</t>
+  </si>
+  <si>
+    <t>Virtue and Valor</t>
+  </si>
+  <si>
+    <t>Adaptive Enchantment</t>
+  </si>
+  <si>
+    <t>Romano &amp; Martin</t>
+  </si>
+  <si>
+    <t>Romano</t>
+  </si>
+  <si>
+    <t>liga-2x2-online-s3-e04</t>
+  </si>
+  <si>
+    <t>Lorehold Spirits</t>
+  </si>
+  <si>
+    <t>Felipe &amp; Pinho</t>
+  </si>
+  <si>
+    <t>Felipe</t>
+  </si>
+  <si>
+    <t>Pinho</t>
+  </si>
+  <si>
+    <t>Explorers of the Deep</t>
+  </si>
+  <si>
+    <t>Guilherme Oliveira</t>
+  </si>
+  <si>
+    <t>Vicente Daye</t>
+  </si>
+  <si>
+    <t>Thiago Cunha &amp; Carlos Spinola</t>
+  </si>
+  <si>
+    <t>Thiago Cunha</t>
+  </si>
+  <si>
+    <t>Carlos Spinola</t>
+  </si>
+  <si>
+    <t>Sneak Attack</t>
+  </si>
+  <si>
+    <t>Mind Flayarrrs</t>
+  </si>
+  <si>
+    <t>Bells</t>
+  </si>
+  <si>
+    <t>Greowty</t>
+  </si>
+  <si>
+    <t>Counter Intelligence</t>
+  </si>
+  <si>
+    <t>Blast from the Past</t>
+  </si>
+  <si>
+    <t>Rafael Silva &amp; Kuka</t>
+  </si>
+  <si>
+    <t>Rafael Silva</t>
+  </si>
+  <si>
+    <t>Kuka</t>
+  </si>
+  <si>
+    <t>liga-2x2-online-s3-e03</t>
+  </si>
+  <si>
+    <t>Silverquill Statement</t>
   </si>
 </sst>
 </file>
@@ -1059,7 +1155,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D99396ED-B3E7-46C7-84C7-4361573AC3B7}">
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr defaultColWidth="19.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
@@ -3781,8 +3877,209 @@
         <v>199</v>
       </c>
     </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>222</v>
+      </c>
+      <c r="B127" t="s">
+        <v>212</v>
+      </c>
+      <c r="C127" t="s">
+        <v>213</v>
+      </c>
+      <c r="D127" t="s">
+        <v>26</v>
+      </c>
+      <c r="E127" t="s">
+        <v>214</v>
+      </c>
+      <c r="F127" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>222</v>
+      </c>
+      <c r="B128" t="s">
+        <v>215</v>
+      </c>
+      <c r="C128" t="s">
+        <v>216</v>
+      </c>
+      <c r="D128" t="s">
+        <v>217</v>
+      </c>
+      <c r="E128" t="s">
+        <v>218</v>
+      </c>
+      <c r="F128" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>222</v>
+      </c>
+      <c r="B129" t="s">
+        <v>220</v>
+      </c>
+      <c r="C129" t="s">
+        <v>221</v>
+      </c>
+      <c r="D129" t="s">
+        <v>22</v>
+      </c>
+      <c r="E129" t="s">
+        <v>137</v>
+      </c>
+      <c r="F129" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>222</v>
+      </c>
+      <c r="B130" t="s">
+        <v>203</v>
+      </c>
+      <c r="C130" t="s">
+        <v>25</v>
+      </c>
+      <c r="D130" t="s">
+        <v>59</v>
+      </c>
+      <c r="E130" t="s">
+        <v>41</v>
+      </c>
+      <c r="F130" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>242</v>
+      </c>
+      <c r="B131" t="s">
+        <v>203</v>
+      </c>
+      <c r="C131" t="s">
+        <v>25</v>
+      </c>
+      <c r="D131" t="s">
+        <v>59</v>
+      </c>
+      <c r="E131" t="s">
+        <v>208</v>
+      </c>
+      <c r="F131" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>242</v>
+      </c>
+      <c r="B132" t="s">
+        <v>224</v>
+      </c>
+      <c r="C132" t="s">
+        <v>225</v>
+      </c>
+      <c r="D132" t="s">
+        <v>226</v>
+      </c>
+      <c r="E132" t="s">
+        <v>227</v>
+      </c>
+      <c r="F132" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>242</v>
+      </c>
+      <c r="B133" t="s">
+        <v>204</v>
+      </c>
+      <c r="C133" t="s">
+        <v>228</v>
+      </c>
+      <c r="D133" t="s">
+        <v>229</v>
+      </c>
+      <c r="E133" t="s">
+        <v>131</v>
+      </c>
+      <c r="F133" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>242</v>
+      </c>
+      <c r="B134" t="s">
+        <v>230</v>
+      </c>
+      <c r="C134" t="s">
+        <v>231</v>
+      </c>
+      <c r="D134" t="s">
+        <v>232</v>
+      </c>
+      <c r="E134" t="s">
+        <v>233</v>
+      </c>
+      <c r="F134" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>242</v>
+      </c>
+      <c r="B135" t="s">
+        <v>132</v>
+      </c>
+      <c r="C135" t="s">
+        <v>235</v>
+      </c>
+      <c r="D135" t="s">
+        <v>236</v>
+      </c>
+      <c r="E135" t="s">
+        <v>237</v>
+      </c>
+      <c r="F135" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>242</v>
+      </c>
+      <c r="B136" t="s">
+        <v>239</v>
+      </c>
+      <c r="C136" t="s">
+        <v>240</v>
+      </c>
+      <c r="D136" t="s">
+        <v>241</v>
+      </c>
+      <c r="E136" t="s">
+        <v>218</v>
+      </c>
+      <c r="F136" t="s">
+        <v>243</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>